<commit_message>
Reference the sample-of-one workpaper (E09) from the Word document
Adds E09 to the evidence references, the workpaper row for each sample
attribute and observation, workpaper references on the exhibits,
conclusion and summary box, and E09 in the workbook's evidence index.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015rwvi2ZZV7Ac5SymUE9zfu
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7_Sample_of_1_MIA25142_Workpaper.xlsx
+++ b/BSI.IT.27.C7_Sample_of_1_MIA25142_Workpaper.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="249">
   <si>
     <t xml:space="preserve">BSI.IT.27.C7 – Network Device Admin Account Review – Sample of One Workpaper (MIA25142)</t>
   </si>
@@ -464,7 +464,7 @@
     <t xml:space="preserve">IAMS Termination Date / Identity Inactive fields; AD 05/15/2026 row 1636; Oct10_2026Users row 1621</t>
   </si>
   <si>
-    <t xml:space="preserve">Evidence index – BSI.IT.27.C7 (E01 – E08)</t>
+    <t xml:space="preserve">Evidence index – BSI.IT.27.C7 (E01 – E09)</t>
   </si>
   <si>
     <t xml:space="preserve">Same references as the "Evidence references" table of the Word document.</t>
@@ -641,6 +641,18 @@
     <t xml:space="preserve">Evidence references</t>
   </si>
   <si>
+    <t xml:space="preserve">E09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSI.IT.27.C7_Sample_of_1_MIA25142_Workpaper.xlsx (this workbook)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample result, attribute testing, evidence map and index for MIA25142</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary box; Section 3 (evidence column, conclusion); Evidence references E09; Exhibits A1-A5</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cross-reference: BSI.IT.27.C7_Design_WT_Sample_of_1_MIA25142.docx → this workbook</t>
   </si>
   <si>
@@ -713,10 +725,10 @@
     <t xml:space="preserve">WP Summary!B9; Sample Attribute Testing (result line)</t>
   </si>
   <si>
-    <t xml:space="preserve">E01-E08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence Index!A5:G12</t>
+    <t xml:space="preserve">E01-E09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence Index!A5:G13</t>
   </si>
   <si>
     <t xml:space="preserve">Exhibit A1</t>
@@ -2220,7 +2232,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -2459,6 +2471,29 @@
       </c>
       <c r="G12" s="6" t="s">
         <v>204</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -2491,31 +2526,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2523,65 +2558,65 @@
         <v>10</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2589,65 +2624,65 @@
         <v>204</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update MIA25142 sample of one (Word + workpaper) for easy evidence tracking
Builds on the tester's edited document (walkthrough attendees and the
Evidence References table are kept): adds a how-to box, extends the
evidence table (E06.10-E06.13 workbook tabs, E09 workpaper), cites the
exact workbook tab and rows for every result, adds a Section 4 evidence
locator, and aligns the result with the attribute matrix: removal within
SLA but not sustained, so the sample fails A6. The workpaper uses the
same E-numbers and result.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015rwvi2ZZV7Ac5SymUE9zfu
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7_Sample_of_1_MIA25142_Workpaper.xlsx
+++ b/BSI.IT.27.C7_Sample_of_1_MIA25142_Workpaper.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="321" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="270">
   <si>
     <t xml:space="preserve">BSI.IT.27.C7 – Network Device Admin Account Review – Sample of One Workpaper (MIA25142)</t>
   </si>
@@ -86,7 +86,7 @@
     <t xml:space="preserve">Design rating</t>
   </si>
   <si>
-    <t xml:space="preserve">Satisfactory (3 observations) – Word doc Section 1</t>
+    <t xml:space="preserve">Satisfactory (4 observations) – Word doc Section 1</t>
   </si>
   <si>
     <t xml:space="preserve">Sample result</t>
@@ -122,7 +122,7 @@
     <t xml:space="preserve">1 Obtain evidence</t>
   </si>
   <si>
-    <t xml:space="preserve">Policies (E01-E03), 2025 Q3 / 2026 Q1 certifications with AD extracts and Netwrix (E04-E05), management response (E06)</t>
+    <t xml:space="preserve">Policies (E01-E03), 2025 Q3 / 2026 Q1 certifications with AD extracts and Netwrix (E04-E05), management response (E07)</t>
   </si>
   <si>
     <t xml:space="preserve">Obtained; ServiceNow ticket not provided (O1)</t>
@@ -158,7 +158,7 @@
     <t xml:space="preserve">Removal by PAM/IAM within 30 business days of the close of the review</t>
   </si>
   <si>
-    <t xml:space="preserve">PASS - 2 business days</t>
+    <t xml:space="preserve">FAIL - removed in 2 business days (within SLA) but back in AD by 11/25/2025</t>
   </si>
   <si>
     <t xml:space="preserve">Section 3 rows 7-8; Exhibit A3</t>
@@ -167,10 +167,10 @@
     <t xml:space="preserve">6-7 Exceptions / escalation</t>
   </si>
   <si>
-    <t xml:space="preserve">No exceptions for this sample; observations recorded</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N/A - observations O1-O3</t>
+    <t xml:space="preserve">Exception record, escalation (PAM Proc. sec. 4.2) and re-grant request for the returned access</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAIL - none provided</t>
   </si>
   <si>
     <t xml:space="preserve">Section 3 rows 9-11</t>
@@ -182,13 +182,16 @@
     <t xml:space="preserve">Control mitigates inappropriate privileged network access for the sample</t>
   </si>
   <si>
+    <t xml:space="preserve">FAIL - access identified as inappropriate was back within 3 months</t>
+  </si>
+  <si>
     <t xml:space="preserve">Section 2 last paragraph; Conclusion</t>
   </si>
   <si>
     <t xml:space="preserve">Conclusion</t>
   </si>
   <si>
-    <t xml:space="preserve">Sample MIA25142 PASSED all control attributes (A1-A6): review initiated by InfoSec, performed by the authorized line manager, inappropriate access revoked and removed by PAM/IAM within the 30-business-day SLA (SUS.IAMS.4.2.5.21). Three observations, no exceptions. Word doc: Section 3 Conclusion.</t>
+    <t xml:space="preserve">Sample MIA25142 FAILED attribute A6 (access stays removed): review initiated by InfoSec, performed by the authorized line manager and documented; access removed on 09/02/2025 within the 30-business-day SLA (SUS.IAMS.4.2.5.21) but back in both groups by 11/25/2025 without a request or escalation (SUS.IAMS.4.2.5.10; PAM Proc. 4.1.1 C4, sec. 4.2), and approved again in 2026 Q1 (A5 - E3). Word doc: Section 3 Conclusion</t>
   </si>
   <si>
     <t xml:space="preserve">Sample MIA25142 – attribute testing against the control description</t>
@@ -221,7 +224,7 @@
     <t xml:space="preserve">2025 Q3 review (launched 08/01/2025) for H2 2025 and 2026 Q1 review (launched 04/09/2026) for H1 2026; MIA25142 included in both</t>
   </si>
   <si>
-    <t xml:space="preserve">E04; E05; E07 tab 2_Step-by-Step 4.1</t>
+    <t xml:space="preserve">E04; E05; E06 tab 2_Step-by-Step 4.1</t>
   </si>
   <si>
     <t xml:space="preserve">Section 3, row 1</t>
@@ -344,6 +347,33 @@
     <t xml:space="preserve">Section 3, row 8; Exhibit A3</t>
   </si>
   <si>
+    <t xml:space="preserve">Access stayed removed - persistence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No - member of both groups again in AD on 11/25/2025; no approved request, Netwrix "member added" event or escalation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E04 AD row 1639; E06 4_Item Detail rows 19, 57; E06 5_Exceptions row 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section 3, row 9; Exhibit A3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026 Q1 review of the re-added access (E3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approved 04/30/2026 without an approved re-grant request</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E05 rows 3260, 3265; E06 4_Item Detail rows 107, 130</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section 3, row 10; Exhibit A4</t>
+  </si>
+  <si>
     <t xml:space="preserve">O1</t>
   </si>
   <si>
@@ -353,10 +383,10 @@
     <t xml:space="preserve">Not provided by management; removal evidenced by Netwrix</t>
   </si>
   <si>
-    <t xml:space="preserve">E07 tab 7_Evidence Status #12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Section 3, row 9</t>
+    <t xml:space="preserve">E06 tab 7_Evidence Status #12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section 3, row 13</t>
   </si>
   <si>
     <t xml:space="preserve">PAM Proc. 4.1.1 C3</t>
@@ -365,16 +395,16 @@
     <t xml:space="preserve">O2</t>
   </si>
   <si>
-    <t xml:space="preserve">Access after removal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Member of both groups again in AD on 11/25/2025; approved by the line manager on 04/30/2026, 07/27/2026 and 08/17/2026. A new grant after a confirmed removal - assessed under SUS.IAMS.4.2.3.4 (provisioning), not this control</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E04 (row 1639); E05 (rows 3260, 3265); E06 (SOX rows 98-100, CyberArk rows 431-433); E07 #5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Section 3, row 10; Exhibits A1, A2, A4</t>
+    <t xml:space="preserve">2026 Q2 status (after the period)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Still approved: SOX Manager 07/27/2026, CyberArk Manager 08/17/2026; AD enabled 10/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E07 / E06 blue tabs: SOX rows 98-100, CyberArk rows 431-433, Oct10_2026Users row 1621; E06 9_Sample Tab Review row 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section 3, row 11; Exhibits A1, A2, A4</t>
   </si>
   <si>
     <t xml:space="preserve">SUS.IAMS.4.2.3.4 (provisioning control)</t>
@@ -383,16 +413,16 @@
     <t xml:space="preserve">O3</t>
   </si>
   <si>
-    <t xml:space="preserve">Account status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IAMS Termination Date 12/31/2024 but Identity Inactive FALSE and AD enabled (11/25/2025, 05/15/2026, 10/10/2026) - termination not evidenced; HR is the authoritative source (SUS.IAMS.4.2.1.1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E04; E05 (row 1636); E06 Oct10_2026Users (row 1621); E07 #4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Section 3, row 11; Exhibits A4, A5</t>
+    <t xml:space="preserve">Account status (E2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAMS Termination Date 12/31/2024, but Identity Inactive FALSE and not excluded as "Terminated in HR" by SanIAM - contract extension pending Fieldglass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E06 tab S13 rows 100-102 vs 192-198; E06 7_Evidence Status #13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Section 3, row 12; Exhibits A3, A5</t>
   </si>
   <si>
     <t xml:space="preserve">SUS.IAMS.4.2.1.1; 4.2.4.3 if HR confirms</t>
@@ -449,19 +479,34 @@
     <t xml:space="preserve">Removal 09/02/2025 vs deadline 10/10/2025; SUS.IAMS.4.2.5.21 (p.22)</t>
   </si>
   <si>
-    <t xml:space="preserve">E07 Testing Walkthrough workbook</t>
+    <t xml:space="preserve">E04 BSI.IT.27.C7.02 Q3_2025.xlsx (AD extract); E06 walkthrough</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AD 11/25/2025 row 1639; 4_Item Detail rows 19, 57 (col V); 5_Exceptions row 8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E05 BSI.IT.27.C7.02 Q1 2026 Cert.xlsx; E06 walkthrough</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rows 3260, 3265; 4_Item Detail rows 107, 130 (col U)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E06 Testing Walkthrough workbook</t>
   </si>
   <si>
     <t xml:space="preserve">Tab 7_Evidence Status #12</t>
   </si>
   <si>
-    <t xml:space="preserve">E04 / E05 / E06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AD 11/25/2025 row 1639; Q1 2026 rows 3260, 3265; C7.Sample SOX rows 98-100, CyberArk rows 431-433; SAMPLE tab screenshots A14, A20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IAMS Termination Date / Identity Inactive fields; AD 05/15/2026 row 1636; Oct10_2026Users row 1621</t>
+    <t xml:space="preserve">E07 C7.Sample.xlsx / E06 blue tabs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOX Manager rows 98-100; CyberArk Manager rows 431-433; Oct10_2026Users row 1621; SAMPLE screenshots A14, A20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E06 tab S13 (SanIAM source)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIA25142 rows 100-102 (not excluded) vs rows 192-198 (excluded - Terminated in HR)</t>
   </si>
   <si>
     <t xml:space="preserve">Evidence index – BSI.IT.27.C7 (E01 – E09)</t>
@@ -584,6 +629,27 @@
     <t xml:space="preserve">E06</t>
   </si>
   <si>
+    <t xml:space="preserve">BSI.IT.27.C7.05 Testing Walkthrough - Combined with 2026 Q2 Sample.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Testing workpaper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10/2026 - IT RCSA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3_Attribute Matrix rows 5-6; 4_Item Detail rows 19, 57, 107, 130; 7_Evidence Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1-A6; O1-O3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence references; closing note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E07</t>
+  </si>
+  <si>
     <t xml:space="preserve">C7.Sample.xlsx (management response)</t>
   </si>
   <si>
@@ -602,27 +668,6 @@
     <t xml:space="preserve">Exhibits A1, A2, A4, A5</t>
   </si>
   <si>
-    <t xml:space="preserve">E07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BSI.IT.27.C7.05 Testing Walkthrough - Combined with 2026 Q2 Sample.xlsx</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Testing workpaper</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10/2026 - IT RCSA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3_Attribute Matrix rows 5-6; 4_Item Detail rows 19, 57, 107, 130; 7_Evidence Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A1-A6; O1-O3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evidence references; closing note</t>
-  </si>
-  <si>
     <t xml:space="preserve">E08</t>
   </si>
   <si>
@@ -707,13 +752,31 @@
     <t xml:space="preserve">Sample Attribute Testing!A5:G12</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Sample of One – rows 9-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Observations O1-O3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sample Attribute Testing!A15:G17</t>
+    <t xml:space="preserve">3. Sample of One – rows 9-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A6 persistence and A5 (E3) – FAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample Attribute Testing!A13:G14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Sample of One – rows 11-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sample Attribute Testing!A17:G19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Evidence Locator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every place MIA25142 appears</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evidence Map; Evidence Index</t>
   </si>
   <si>
     <t xml:space="preserve">3. Conclusion</t>
@@ -737,7 +800,7 @@
     <t xml:space="preserve">2026 Q2 SOX Manager certification screenshot (rows 98-100)</t>
   </si>
   <si>
-    <t xml:space="preserve">Evidence Map (O2); Evidence Index E06</t>
+    <t xml:space="preserve">Evidence Map (O2); Evidence Index E07</t>
   </si>
   <si>
     <t xml:space="preserve">Exhibit A2</t>
@@ -761,7 +824,7 @@
     <t xml:space="preserve">Account and access status after the revocation</t>
   </si>
   <si>
-    <t xml:space="preserve">Evidence Map (O2, O3); Evidence Index E05, E06</t>
+    <t xml:space="preserve">Evidence Map (O2, O3); Evidence Index E05, E07</t>
   </si>
   <si>
     <t xml:space="preserve">Exhibit A5</t>
@@ -770,7 +833,7 @@
     <t xml:space="preserve">AD user export command screenshot</t>
   </si>
   <si>
-    <t xml:space="preserve">Evidence Map (O3); Evidence Index E06</t>
+    <t xml:space="preserve">Evidence Map (O3); Evidence Index E07</t>
   </si>
 </sst>
 </file>
@@ -842,7 +905,7 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF006100"/>
+      <color rgb="FF9C0006"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -856,7 +919,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -890,7 +953,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
-        <bgColor rgb="FFFFCC99"/>
+        <bgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -980,7 +1049,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -996,15 +1065,15 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1031,7 +1100,7 @@
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF9C0006"/>
       <rgbColor rgb="FF006100"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
@@ -1062,7 +1131,7 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFC7CE"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -1330,20 +1399,20 @@
         <v>9</v>
       </c>
       <c r="E4" s="6" t="n">
-        <f aca="false">COUNTA('Sample Attribute Testing'!E5:E12)</f>
-        <v>8</v>
+        <f aca="false">COUNTA('Sample Attribute Testing'!E5:E14)</f>
+        <v>10</v>
       </c>
       <c r="F4" s="6" t="n">
-        <f aca="false">COUNTIF('Sample Attribute Testing'!E5:E12,"PASS")</f>
+        <f aca="false">COUNTIF('Sample Attribute Testing'!E5:E14,"PASS")</f>
         <v>8</v>
       </c>
       <c r="G4" s="6" t="n">
         <f aca="false">E4-F4</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H4" s="7" t="str">
         <f aca="false">IF(G4=0,"PASS","FAIL")</f>
-        <v>PASS</v>
+        <v>FAIL</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="72" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1384,7 +1453,7 @@
         <v>15</v>
       </c>
       <c r="E6" s="6" t="n">
-        <f aca="false">COUNTA('Sample Attribute Testing'!A15:A17)</f>
+        <f aca="false">COUNTA('Sample Attribute Testing'!A17:A19)</f>
         <v>3</v>
       </c>
       <c r="F6" s="6" t="n">
@@ -1419,8 +1488,8 @@
         <v>21</v>
       </c>
       <c r="B9" s="9" t="str">
-        <f aca="false">IF(COUNTIF('Sample Attribute Testing'!E5:E12,"PASS")=COUNTA('Sample Attribute Testing'!E5:E12),"PASS – all attributes met","FAIL")</f>
-        <v>PASS – all attributes met</v>
+        <f aca="false">IF(COUNTIF('Sample Attribute Testing'!E5:E14,"PASS")=COUNTA('Sample Attribute Testing'!E5:E14),"PASS – all attributes met","FAIL")</f>
+        <v>FAIL</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1531,12 +1600,12 @@
         <v>43</v>
       </c>
       <c r="C18" s="6"/>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
       <c r="H18" s="6" t="s">
         <v>45</v>
       </c>
@@ -1549,12 +1618,12 @@
         <v>47</v>
       </c>
       <c r="C19" s="6"/>
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
       <c r="H19" s="6" t="s">
         <v>49</v>
       </c>
@@ -1567,29 +1636,29 @@
         <v>51</v>
       </c>
       <c r="C20" s="6"/>
-      <c r="D20" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
+      <c r="D20" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
       <c r="H20" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B22" s="15" t="s">
+      <c r="A22" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
+      <c r="B22" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -1625,7 +1694,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -1639,7 +1708,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1650,7 +1719,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1661,16 +1730,16 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>29</v>
@@ -1679,291 +1748,337 @@
         <v>30</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E5" s="12" t="s">
         <v>37</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E6" s="12" t="s">
         <v>37</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>37</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E8" s="12" t="s">
         <v>37</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E9" s="12" t="s">
         <v>37</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E10" s="12" t="s">
         <v>37</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E11" s="12" t="s">
         <v>37</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E12" s="12" t="s">
         <v>37</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-    </row>
-    <row r="15" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>117</v>
-      </c>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="D17" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="E17" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="G17" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="E17" s="13" t="s">
+    </row>
+    <row r="18" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="E18" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="16" t="str">
-        <f aca="false">"Sample result: "&amp;IF(COUNTIF(E5:E12,"PASS")=COUNTA(E5:E12),"PASS","FAIL")&amp;" – "&amp;COUNTIF(E5:E12,"PASS")&amp;" of "&amp;COUNTA(E5:E12)&amp;" attribute checks passed; "&amp;COUNTA(A15:A17)&amp;" observations."</f>
-        <v>Sample result: PASS – 8 of 8 attribute checks passed; 3 observations.</v>
-      </c>
-      <c r="B19" s="16"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
+      <c r="F18" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="16" t="str">
+        <f aca="false">"Sample result: "&amp;IF(COUNTIF(E5:E14,"PASS")=COUNTA(E5:E14),"PASS","FAIL")&amp;" – "&amp;COUNTIF(E5:E14,"PASS")&amp;" of "&amp;COUNTA(E5:E14)&amp;" attribute checks passed; "&amp;COUNTA(A17:A19)&amp;" observations."</f>
+        <v>Sample result: FAIL – 8 of 10 attribute checks passed; 3 observations.</v>
+      </c>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A21:G21"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1980,7 +2095,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -1992,7 +2107,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2001,7 +2116,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2010,16 +2125,16 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="E4" s="4" t="s">
         <v>30</v>
@@ -2027,189 +2142,223 @@
     </row>
     <row r="5" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>107</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>113</v>
-      </c>
       <c r="C14" s="6" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="E15" s="6" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11" t="s">
         <v>122</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -2246,7 +2395,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2257,7 +2406,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2268,22 +2417,22 @@
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>149</v>
+        <v>164</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>150</v>
+        <v>165</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>151</v>
+        <v>166</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>152</v>
+        <v>167</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>30</v>
@@ -2291,209 +2440,209 @@
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>154</v>
+        <v>169</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>159</v>
+        <v>174</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>160</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>28</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>160</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>173</v>
+        <v>188</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>202</v>
+        <v>217</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="F13" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>197</v>
-      </c>
       <c r="G13" s="6" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>
@@ -2516,7 +2665,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -2526,31 +2675,31 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>211</v>
+        <v>226</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>215</v>
+        <v>230</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2558,131 +2707,153 @@
         <v>10</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>216</v>
+        <v>231</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>227</v>
+        <v>242</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>228</v>
+        <v>243</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>230</v>
+        <v>245</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>231</v>
+        <v>246</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>234</v>
+        <v>250</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>235</v>
+        <v>251</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>236</v>
+        <v>252</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>237</v>
+        <v>253</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>238</v>
+        <v>219</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>237</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>240</v>
+        <v>256</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>241</v>
+        <v>257</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>242</v>
+        <v>258</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>243</v>
+        <v>259</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>244</v>
+        <v>260</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>246</v>
+        <v>261</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>248</v>
+        <v>263</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>269</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add BSI.IT.27.C7 evidence package (folder + zip) with E00 index
Every referenced file is renamed by its E-number (BSI.IT.27.C7_E##_...)
and indexed with MD5 in BSI.IT.27.C7_E00_Evidence Index.xlsx; the
SanIAM CSVs sit in BSI.IT.27.C7_E06.12_SanIAM source files. The sample
of one Word document and workpaper now cite these package file names.
E01a (IAM v10.0), E03, E04 and E05 were not provided and are flagged
in the index for adding from the original walkthrough folder.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015rwvi2ZZV7Ac5SymUE9zfu
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7_Sample_of_1_MIA25142_Workpaper.xlsx
+++ b/BSI.IT.27.C7_Sample_of_1_MIA25142_Workpaper.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">BSI.IT.27.C7 – Network Device Admin Account Review – Sample of One Workpaper (MIA25142)</t>
   </si>
   <si>
-    <t xml:space="preserve">Supports the Word document "BSI.IT.27.C7_Design_WT_Sample_of_1_MIA25142.docx". Each row gives the matching section / exhibit of that document.</t>
+    <t xml:space="preserve">Supports the Word document "BSI.IT.27.C7_Design_WT_Sample_of_1_MIA25142.docx (folder BSI.IT.27.C7)". Each row gives the matching section / exhibit of that document.</t>
   </si>
   <si>
     <t xml:space="preserve">KPI</t>
@@ -95,7 +95,7 @@
     <t xml:space="preserve">Word document</t>
   </si>
   <si>
-    <t xml:space="preserve">BSI.IT.27.C7_Design_WT_Sample_of_1_MIA25142.docx</t>
+    <t xml:space="preserve">BSI.IT.27.C7_Design_WT_Sample_of_1_MIA25142.docx (folder BSI.IT.27.C7)</t>
   </si>
   <si>
     <t xml:space="preserve">Walkthrough</t>
@@ -536,7 +536,7 @@
     <t xml:space="preserve">E01</t>
   </si>
   <si>
-    <t xml:space="preserve">CUSO Identity and Access Management Standard v11.0 (BSIIT21.PDF)</t>
+    <t xml:space="preserve">BSI.IT.27.C7_E01_IAM Standard v11.0 (BSIIT21).pdf</t>
   </si>
   <si>
     <t xml:space="preserve">Policy</t>
@@ -557,7 +557,7 @@
     <t xml:space="preserve">E02</t>
   </si>
   <si>
-    <t xml:space="preserve">PAM Recertification Procedure (BSI) 04.22.26.pdf (v2.0)</t>
+    <t xml:space="preserve">BSI.IT.27.C7_E02_PAM Recertification Procedure (BSI) 04.22.26.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">04/22/2026 - BSI CISO</t>
@@ -572,7 +572,7 @@
     <t xml:space="preserve">E03</t>
   </si>
   <si>
-    <t xml:space="preserve">BSI.IT.27.C7.03 PAM Definition of Privilege.pdf (v10.0)</t>
+    <t xml:space="preserve">BSI.IT.27.C7_E03_PAM Definition of Privilege.pdf (not in package)</t>
   </si>
   <si>
     <t xml:space="preserve">03/11/2025</t>
@@ -587,7 +587,7 @@
     <t xml:space="preserve">E04</t>
   </si>
   <si>
-    <t xml:space="preserve">BSI.IT.27.C7.02 Q3_2025.xlsx</t>
+    <t xml:space="preserve">BSI.IT.27.C7_E04_Q3_2025.xlsx (not in package)</t>
   </si>
   <si>
     <t xml:space="preserve">SailPoint export, AD extract, Netwrix log</t>
@@ -608,7 +608,7 @@
     <t xml:space="preserve">E05</t>
   </si>
   <si>
-    <t xml:space="preserve">BSI.IT.27.C7.02 Q1 2026 Cert.xlsx</t>
+    <t xml:space="preserve">BSI.IT.27.C7_E05_Q1 2026 Cert.xlsx (not in package)</t>
   </si>
   <si>
     <t xml:space="preserve">SailPoint export, AD extract</t>
@@ -629,7 +629,7 @@
     <t xml:space="preserve">E06</t>
   </si>
   <si>
-    <t xml:space="preserve">BSI.IT.27.C7.05 Testing Walkthrough - Combined with 2026 Q2 Sample.xlsx</t>
+    <t xml:space="preserve">BSI.IT.27.C7_E06_Testing Walkthrough - Combined with 2026 Q2 Sample.xlsx</t>
   </si>
   <si>
     <t xml:space="preserve">Testing workpaper</t>
@@ -650,7 +650,7 @@
     <t xml:space="preserve">E07</t>
   </si>
   <si>
-    <t xml:space="preserve">C7.Sample.xlsx (management response)</t>
+    <t xml:space="preserve">BSI.IT.27.C7_E07_C7.Sample.xlsx</t>
   </si>
   <si>
     <t xml:space="preserve">SailPoint exports, AD user export, screenshots</t>
@@ -671,7 +671,7 @@
     <t xml:space="preserve">E08</t>
   </si>
   <si>
-    <t xml:space="preserve">Sample step taken.docx</t>
+    <t xml:space="preserve">BSI.IT.27.C7_E08_Sample step taken.docx</t>
   </si>
   <si>
     <t xml:space="preserve">Request</t>
@@ -689,7 +689,7 @@
     <t xml:space="preserve">E09</t>
   </si>
   <si>
-    <t xml:space="preserve">BSI.IT.27.C7_Sample_of_1_MIA25142_Workpaper.xlsx (this workbook)</t>
+    <t xml:space="preserve">BSI.IT.27.C7_E09_Sample of 1 MIA25142 Workpaper.xlsx (this workbook)</t>
   </si>
   <si>
     <t xml:space="preserve">Sample result, attribute testing, evidence map and index for MIA25142</t>
@@ -698,7 +698,7 @@
     <t xml:space="preserve">Summary box; Section 3 (evidence column, conclusion); Evidence references E09; Exhibits A1-A5</t>
   </si>
   <si>
-    <t xml:space="preserve">Cross-reference: BSI.IT.27.C7_Design_WT_Sample_of_1_MIA25142.docx → this workbook</t>
+    <t xml:space="preserve">Cross-reference: BSI.IT.27.C7_Design_WT_Sample_of_1_MIA25142.docx (folder BSI.IT.27.C7) → this workbook</t>
   </si>
   <si>
     <t xml:space="preserve">Word document section / exhibit</t>

</xml_diff>